<commit_message>
Refine app version update workflows
</commit_message>
<xml_diff>
--- a/outputs/app-version-update-description-template/APP更新描述模板.xlsx
+++ b/outputs/app-version-update-description-template/APP更新描述模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新描述模板" sheetId="1" r:id="Rdccb7b054bcb4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新描述模板" sheetId="1" r:id="Ra3ab03c7dd6d4907"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,12 +30,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2686F6"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -63,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -85,6 +90,19 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -290,6 +308,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -299,114 +318,135 @@
       <x:c r="B1" s="8" t="str">
         <x:v>更新描述</x:v>
       </x:c>
+      <x:c r="C1" s="14" t="str">
+        <x:v>APP 强制更新描述</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="9" t="str">
         <x:v>中文</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str"/>
+      <x:c r="C2" s="16" t="str"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="9" t="str">
         <x:v>英语</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str"/>
+      <x:c r="C3" s="16" t="str"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="9" t="str">
         <x:v>繁体中文</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str"/>
+      <x:c r="C4" s="16" t="str"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="9" t="str">
         <x:v>德语</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str"/>
+      <x:c r="C5" s="16" t="str"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>法语</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str"/>
+      <x:c r="C6" s="16" t="str"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="9" t="str">
         <x:v>日语</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str"/>
+      <x:c r="C7" s="16" t="str"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>西班牙语</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str"/>
+      <x:c r="C8" s="16" t="str"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="9" t="str">
         <x:v>阿拉伯语</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str"/>
+      <x:c r="C9" s="16" t="str"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>捷克语</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str"/>
+      <x:c r="C10" s="16" t="str"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="9" t="str">
         <x:v>波兰语</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str"/>
+      <x:c r="C11" s="16" t="str"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="9" t="str">
         <x:v>土耳其语</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str"/>
+      <x:c r="C12" s="16" t="str"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="9" t="str">
         <x:v>芬兰语</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str"/>
+      <x:c r="C13" s="16" t="str"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="9" t="str">
         <x:v>意大利语</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str"/>
+      <x:c r="C14" s="16" t="str"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="9" t="str">
         <x:v>匈牙利语</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str"/>
+      <x:c r="C15" s="16" t="str"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="9" t="str">
         <x:v>罗马尼亚语</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str"/>
+      <x:c r="C16" s="16" t="str"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="9" t="str">
         <x:v>韩语</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str"/>
+      <x:c r="C17" s="16" t="str"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>立陶宛语</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str"/>
+      <x:c r="C18" s="16" t="str"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="9" t="str">
         <x:v>马来语</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str"/>
+      <x:c r="C19" s="16" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update version upgrade prototype and documentation
</commit_message>
<xml_diff>
--- a/outputs/app-version-update-description-template/APP更新描述模板.xlsx
+++ b/outputs/app-version-update-description-template/APP更新描述模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新描述模板" sheetId="1" r:id="Ra3ab03c7dd6d4907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新描述模板" sheetId="1" r:id="R9f49d599279c4e03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -316,137 +316,135 @@
         <x:v>语种</x:v>
       </x:c>
       <x:c r="B1" s="8" t="str">
-        <x:v>更新描述</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>APP 强制更新描述</x:v>
-      </x:c>
+        <x:v>版本描述</x:v>
+      </x:c>
+      <x:c r="C1"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="9" t="str">
         <x:v>中文</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str"/>
-      <x:c r="C2" s="16" t="str"/>
+      <x:c r="C2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="9" t="str">
         <x:v>英语</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str"/>
-      <x:c r="C3" s="16" t="str"/>
+      <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="9" t="str">
         <x:v>繁体中文</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str"/>
-      <x:c r="C4" s="16" t="str"/>
+      <x:c r="C4"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="9" t="str">
         <x:v>德语</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str"/>
-      <x:c r="C5" s="16" t="str"/>
+      <x:c r="C5"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>法语</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str"/>
-      <x:c r="C6" s="16" t="str"/>
+      <x:c r="C6"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="9" t="str">
         <x:v>日语</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str"/>
-      <x:c r="C7" s="16" t="str"/>
+      <x:c r="C7"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>西班牙语</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str"/>
-      <x:c r="C8" s="16" t="str"/>
+      <x:c r="C8"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="9" t="str">
         <x:v>阿拉伯语</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str"/>
-      <x:c r="C9" s="16" t="str"/>
+      <x:c r="C9"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>捷克语</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str"/>
-      <x:c r="C10" s="16" t="str"/>
+      <x:c r="C10"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="9" t="str">
         <x:v>波兰语</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str"/>
-      <x:c r="C11" s="16" t="str"/>
+      <x:c r="C11"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="9" t="str">
         <x:v>土耳其语</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str"/>
-      <x:c r="C12" s="16" t="str"/>
+      <x:c r="C12"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="9" t="str">
         <x:v>芬兰语</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str"/>
-      <x:c r="C13" s="16" t="str"/>
+      <x:c r="C13"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="9" t="str">
         <x:v>意大利语</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str"/>
-      <x:c r="C14" s="16" t="str"/>
+      <x:c r="C14"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="9" t="str">
         <x:v>匈牙利语</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str"/>
-      <x:c r="C15" s="16" t="str"/>
+      <x:c r="C15"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="9" t="str">
         <x:v>罗马尼亚语</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str"/>
-      <x:c r="C16" s="16" t="str"/>
+      <x:c r="C16"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="9" t="str">
         <x:v>韩语</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str"/>
-      <x:c r="C17" s="16" t="str"/>
+      <x:c r="C17"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>立陶宛语</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str"/>
-      <x:c r="C18" s="16" t="str"/>
+      <x:c r="C18"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="9" t="str">
         <x:v>马来语</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str"/>
-      <x:c r="C19" s="16" t="str"/>
+      <x:c r="C19"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>